<commit_message>
Add 3-way role comparison sheet for site patrol inspections
Adds a 3자_역할비교 sheet comparing 안전보건관리책임자, 안전관리자, and
관리감독자 roles during the management-responsible person's site patrol
inspection (scope, patrol role, reporting content, response to findings,
authority, legal basis).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SqkinqfGqqfBrcHRBkScVm
</commit_message>
<xml_diff>
--- a/templates/본사현장_안전관리조직도.xlsx
+++ b/templates/본사현장_안전관리조직도.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet name="안전관리조직도" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="책임과권한" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3자_역할비교" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'안전관리조직도'!$A$1:$AF$45</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'책임과권한'!$A$1:$AF$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'3자_역할비교'!$A$1:$AH$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,6 +106,23 @@
       <color rgb="FF595959"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="FF000000"/>
+      <sz val="9.300000000000001"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <i val="1"/>
+      <color rgb="FF595959"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -133,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -322,11 +341,55 @@
         <color rgb="FFBFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -393,6 +456,18 @@
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1377,6 +1452,577 @@
           <t>경영책임자 현장순회점검 시 책임과 권한</t>
         </is>
       </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>(현장소장(안전보건관리책임자) 및 안전관리자 - 산업안전보건법 제15조·제17조, 중대재해처벌법 시행령 제4조 기준)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="10" customHeight="1"/>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>1. 현장소장 (안전보건관리책임자) - 현장 총괄·최종 의사결정자</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="C6" s="36" t="n"/>
+      <c r="D6" s="36" t="n"/>
+      <c r="E6" s="36" t="n"/>
+      <c r="F6" s="36" t="n"/>
+      <c r="G6" s="37" t="n"/>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+      <c r="I6" s="36" t="n"/>
+      <c r="J6" s="36" t="n"/>
+      <c r="K6" s="36" t="n"/>
+      <c r="L6" s="36" t="n"/>
+      <c r="M6" s="36" t="n"/>
+      <c r="N6" s="36" t="n"/>
+      <c r="O6" s="36" t="n"/>
+      <c r="P6" s="36" t="n"/>
+      <c r="Q6" s="36" t="n"/>
+      <c r="R6" s="36" t="n"/>
+      <c r="S6" s="36" t="n"/>
+      <c r="T6" s="36" t="n"/>
+      <c r="U6" s="36" t="n"/>
+      <c r="V6" s="36" t="n"/>
+      <c r="W6" s="36" t="n"/>
+      <c r="X6" s="36" t="n"/>
+      <c r="Y6" s="36" t="n"/>
+      <c r="Z6" s="36" t="n"/>
+      <c r="AA6" s="36" t="n"/>
+      <c r="AB6" s="36" t="n"/>
+      <c r="AC6" s="36" t="n"/>
+      <c r="AD6" s="36" t="n"/>
+      <c r="AE6" s="36" t="n"/>
+      <c r="AF6" s="37" t="n"/>
+    </row>
+    <row r="7" ht="95" customHeight="1">
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>책임</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="n"/>
+      <c r="D7" s="36" t="n"/>
+      <c r="E7" s="36" t="n"/>
+      <c r="F7" s="36" t="n"/>
+      <c r="G7" s="37" t="n"/>
+      <c r="H7" s="31" t="inlineStr">
+        <is>
+          <t>- 현장 전체 안전보건관리에 대한 총괄 책임 - 순회점검 시 안전보건관리체계 이행현황(위험성평가, 교육, 관리비 집행 등)을 사실대로 보고
+- 점검 중 지적된 위험요인·미비사항에 대한 시정조치 및 재발방지대책 수립·이행
+- 점검결과에 따른 후속조치 이행 여부를 경영책임자에게 사후 보고
+- 근로자 의견청취 결과를 안전보건관리체계에 반영
+- 협력업체(수급인) 포함 현장 전체의 산업안전보건법 제15조 법정업무 이행</t>
+        </is>
+      </c>
+      <c r="I7" s="36" t="n"/>
+      <c r="J7" s="36" t="n"/>
+      <c r="K7" s="36" t="n"/>
+      <c r="L7" s="36" t="n"/>
+      <c r="M7" s="36" t="n"/>
+      <c r="N7" s="36" t="n"/>
+      <c r="O7" s="36" t="n"/>
+      <c r="P7" s="36" t="n"/>
+      <c r="Q7" s="36" t="n"/>
+      <c r="R7" s="36" t="n"/>
+      <c r="S7" s="36" t="n"/>
+      <c r="T7" s="36" t="n"/>
+      <c r="U7" s="36" t="n"/>
+      <c r="V7" s="36" t="n"/>
+      <c r="W7" s="36" t="n"/>
+      <c r="X7" s="36" t="n"/>
+      <c r="Y7" s="36" t="n"/>
+      <c r="Z7" s="36" t="n"/>
+      <c r="AA7" s="36" t="n"/>
+      <c r="AB7" s="36" t="n"/>
+      <c r="AC7" s="36" t="n"/>
+      <c r="AD7" s="36" t="n"/>
+      <c r="AE7" s="36" t="n"/>
+      <c r="AF7" s="37" t="n"/>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>권한</t>
+        </is>
+      </c>
+      <c r="C8" s="36" t="n"/>
+      <c r="D8" s="36" t="n"/>
+      <c r="E8" s="36" t="n"/>
+      <c r="F8" s="36" t="n"/>
+      <c r="G8" s="37" t="n"/>
+      <c r="H8" s="31" t="inlineStr">
+        <is>
+          <t>- 현장 내 안전보건 관련 사항에 대한 최종 의사결정권
+- 위험 발생·우려 시 작업중지 명령권
+- 안전관리자 등 안전보건 인력에 대한 지휘·감독권
+- 협력업체에 대한 관리·감독 및 시정지시권
+- 안전보건관리비 집행 승인권</t>
+        </is>
+      </c>
+      <c r="I8" s="36" t="n"/>
+      <c r="J8" s="36" t="n"/>
+      <c r="K8" s="36" t="n"/>
+      <c r="L8" s="36" t="n"/>
+      <c r="M8" s="36" t="n"/>
+      <c r="N8" s="36" t="n"/>
+      <c r="O8" s="36" t="n"/>
+      <c r="P8" s="36" t="n"/>
+      <c r="Q8" s="36" t="n"/>
+      <c r="R8" s="36" t="n"/>
+      <c r="S8" s="36" t="n"/>
+      <c r="T8" s="36" t="n"/>
+      <c r="U8" s="36" t="n"/>
+      <c r="V8" s="36" t="n"/>
+      <c r="W8" s="36" t="n"/>
+      <c r="X8" s="36" t="n"/>
+      <c r="Y8" s="36" t="n"/>
+      <c r="Z8" s="36" t="n"/>
+      <c r="AA8" s="36" t="n"/>
+      <c r="AB8" s="36" t="n"/>
+      <c r="AC8" s="36" t="n"/>
+      <c r="AD8" s="36" t="n"/>
+      <c r="AE8" s="36" t="n"/>
+      <c r="AF8" s="37" t="n"/>
+    </row>
+    <row r="9" ht="12" customHeight="1"/>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2. 안전관리자 - 기술 전문가·보좌기관</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="C11" s="36" t="n"/>
+      <c r="D11" s="36" t="n"/>
+      <c r="E11" s="36" t="n"/>
+      <c r="F11" s="36" t="n"/>
+      <c r="G11" s="37" t="n"/>
+      <c r="H11" s="27" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+      <c r="I11" s="36" t="n"/>
+      <c r="J11" s="36" t="n"/>
+      <c r="K11" s="36" t="n"/>
+      <c r="L11" s="36" t="n"/>
+      <c r="M11" s="36" t="n"/>
+      <c r="N11" s="36" t="n"/>
+      <c r="O11" s="36" t="n"/>
+      <c r="P11" s="36" t="n"/>
+      <c r="Q11" s="36" t="n"/>
+      <c r="R11" s="36" t="n"/>
+      <c r="S11" s="36" t="n"/>
+      <c r="T11" s="36" t="n"/>
+      <c r="U11" s="36" t="n"/>
+      <c r="V11" s="36" t="n"/>
+      <c r="W11" s="36" t="n"/>
+      <c r="X11" s="36" t="n"/>
+      <c r="Y11" s="36" t="n"/>
+      <c r="Z11" s="36" t="n"/>
+      <c r="AA11" s="36" t="n"/>
+      <c r="AB11" s="36" t="n"/>
+      <c r="AC11" s="36" t="n"/>
+      <c r="AD11" s="36" t="n"/>
+      <c r="AE11" s="36" t="n"/>
+      <c r="AF11" s="37" t="n"/>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>책임</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="n"/>
+      <c r="D12" s="36" t="n"/>
+      <c r="E12" s="36" t="n"/>
+      <c r="F12" s="36" t="n"/>
+      <c r="G12" s="37" t="n"/>
+      <c r="H12" s="31" t="inlineStr">
+        <is>
+          <t>- 안전에 관한 기술적 사항에 대해 안전보건관리책임자를 보좌
+- 관리감독자에게 안전 관련 지도·조언
+- 순회점검 시 위험성평가 결과, 안전장치·보호구 점검현황, 아차사고/재해 통계 등 전문분야 자료 준비·설명
+- 지적사항 중 기술적 사항에 대한 개선방안 제시
+- 사업장 순회점검, 안전교육계획 수립, 산재 원인조사 등 법정 고유업무 수행(시행령 별표3)</t>
+        </is>
+      </c>
+      <c r="I12" s="36" t="n"/>
+      <c r="J12" s="36" t="n"/>
+      <c r="K12" s="36" t="n"/>
+      <c r="L12" s="36" t="n"/>
+      <c r="M12" s="36" t="n"/>
+      <c r="N12" s="36" t="n"/>
+      <c r="O12" s="36" t="n"/>
+      <c r="P12" s="36" t="n"/>
+      <c r="Q12" s="36" t="n"/>
+      <c r="R12" s="36" t="n"/>
+      <c r="S12" s="36" t="n"/>
+      <c r="T12" s="36" t="n"/>
+      <c r="U12" s="36" t="n"/>
+      <c r="V12" s="36" t="n"/>
+      <c r="W12" s="36" t="n"/>
+      <c r="X12" s="36" t="n"/>
+      <c r="Y12" s="36" t="n"/>
+      <c r="Z12" s="36" t="n"/>
+      <c r="AA12" s="36" t="n"/>
+      <c r="AB12" s="36" t="n"/>
+      <c r="AC12" s="36" t="n"/>
+      <c r="AD12" s="36" t="n"/>
+      <c r="AE12" s="36" t="n"/>
+      <c r="AF12" s="37" t="n"/>
+    </row>
+    <row r="13" ht="68" customHeight="1">
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>권한</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="n"/>
+      <c r="D13" s="36" t="n"/>
+      <c r="E13" s="36" t="n"/>
+      <c r="F13" s="36" t="n"/>
+      <c r="G13" s="37" t="n"/>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>- 위험 발견 시 안전보건관리책임자(또는 사업주)에게 작업중지 요청권
+- 관리감독자에 대한 지도·조언권
+- 안전보건 관련 자료 열람 및 시정요구권
+- 업무수행에 필요한 권한·시설·장비를 사업주로부터 지원받을 권리(법 제18조 - 독립적 업무수행 보장)</t>
+        </is>
+      </c>
+      <c r="I13" s="36" t="n"/>
+      <c r="J13" s="36" t="n"/>
+      <c r="K13" s="36" t="n"/>
+      <c r="L13" s="36" t="n"/>
+      <c r="M13" s="36" t="n"/>
+      <c r="N13" s="36" t="n"/>
+      <c r="O13" s="36" t="n"/>
+      <c r="P13" s="36" t="n"/>
+      <c r="Q13" s="36" t="n"/>
+      <c r="R13" s="36" t="n"/>
+      <c r="S13" s="36" t="n"/>
+      <c r="T13" s="36" t="n"/>
+      <c r="U13" s="36" t="n"/>
+      <c r="V13" s="36" t="n"/>
+      <c r="W13" s="36" t="n"/>
+      <c r="X13" s="36" t="n"/>
+      <c r="Y13" s="36" t="n"/>
+      <c r="Z13" s="36" t="n"/>
+      <c r="AA13" s="36" t="n"/>
+      <c r="AB13" s="36" t="n"/>
+      <c r="AC13" s="36" t="n"/>
+      <c r="AD13" s="36" t="n"/>
+      <c r="AE13" s="36" t="n"/>
+      <c r="AF13" s="37" t="n"/>
+    </row>
+    <row r="14" ht="12" customHeight="1"/>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>3. 핵심 비교</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="C16" s="36" t="n"/>
+      <c r="D16" s="36" t="n"/>
+      <c r="E16" s="36" t="n"/>
+      <c r="F16" s="36" t="n"/>
+      <c r="G16" s="36" t="n"/>
+      <c r="H16" s="36" t="n"/>
+      <c r="I16" s="37" t="n"/>
+      <c r="J16" s="27" t="inlineStr">
+        <is>
+          <t>현장소장(안전보건관리책임자)</t>
+        </is>
+      </c>
+      <c r="K16" s="36" t="n"/>
+      <c r="L16" s="36" t="n"/>
+      <c r="M16" s="36" t="n"/>
+      <c r="N16" s="36" t="n"/>
+      <c r="O16" s="36" t="n"/>
+      <c r="P16" s="36" t="n"/>
+      <c r="Q16" s="36" t="n"/>
+      <c r="R16" s="36" t="n"/>
+      <c r="S16" s="37" t="n"/>
+      <c r="T16" s="27" t="inlineStr">
+        <is>
+          <t>안전관리자</t>
+        </is>
+      </c>
+      <c r="U16" s="36" t="n"/>
+      <c r="V16" s="36" t="n"/>
+      <c r="W16" s="36" t="n"/>
+      <c r="X16" s="36" t="n"/>
+      <c r="Y16" s="36" t="n"/>
+      <c r="Z16" s="36" t="n"/>
+      <c r="AA16" s="36" t="n"/>
+      <c r="AB16" s="36" t="n"/>
+      <c r="AC16" s="36" t="n"/>
+      <c r="AD16" s="36" t="n"/>
+      <c r="AE16" s="36" t="n"/>
+      <c r="AF16" s="37" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>성격</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="36" t="n"/>
+      <c r="F17" s="36" t="n"/>
+      <c r="G17" s="36" t="n"/>
+      <c r="H17" s="36" t="n"/>
+      <c r="I17" s="37" t="n"/>
+      <c r="J17" s="34" t="inlineStr">
+        <is>
+          <t>현장 총괄·최종 의사결정자</t>
+        </is>
+      </c>
+      <c r="K17" s="36" t="n"/>
+      <c r="L17" s="36" t="n"/>
+      <c r="M17" s="36" t="n"/>
+      <c r="N17" s="36" t="n"/>
+      <c r="O17" s="36" t="n"/>
+      <c r="P17" s="36" t="n"/>
+      <c r="Q17" s="36" t="n"/>
+      <c r="R17" s="36" t="n"/>
+      <c r="S17" s="37" t="n"/>
+      <c r="T17" s="34" t="inlineStr">
+        <is>
+          <t>기술 전문가·보좌기관</t>
+        </is>
+      </c>
+      <c r="U17" s="36" t="n"/>
+      <c r="V17" s="36" t="n"/>
+      <c r="W17" s="36" t="n"/>
+      <c r="X17" s="36" t="n"/>
+      <c r="Y17" s="36" t="n"/>
+      <c r="Z17" s="36" t="n"/>
+      <c r="AA17" s="36" t="n"/>
+      <c r="AB17" s="36" t="n"/>
+      <c r="AC17" s="36" t="n"/>
+      <c r="AD17" s="36" t="n"/>
+      <c r="AE17" s="36" t="n"/>
+      <c r="AF17" s="37" t="n"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>순회점검 역할</t>
+        </is>
+      </c>
+      <c r="C18" s="36" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="36" t="n"/>
+      <c r="F18" s="36" t="n"/>
+      <c r="G18" s="36" t="n"/>
+      <c r="H18" s="36" t="n"/>
+      <c r="I18" s="37" t="n"/>
+      <c r="J18" s="34" t="inlineStr">
+        <is>
+          <t>전체 현황 보고 + 최종 책임</t>
+        </is>
+      </c>
+      <c r="K18" s="36" t="n"/>
+      <c r="L18" s="36" t="n"/>
+      <c r="M18" s="36" t="n"/>
+      <c r="N18" s="36" t="n"/>
+      <c r="O18" s="36" t="n"/>
+      <c r="P18" s="36" t="n"/>
+      <c r="Q18" s="36" t="n"/>
+      <c r="R18" s="36" t="n"/>
+      <c r="S18" s="37" t="n"/>
+      <c r="T18" s="34" t="inlineStr">
+        <is>
+          <t>전문분야(위험성평가·점검기록) 설명 + 기술적 개선안 제시</t>
+        </is>
+      </c>
+      <c r="U18" s="36" t="n"/>
+      <c r="V18" s="36" t="n"/>
+      <c r="W18" s="36" t="n"/>
+      <c r="X18" s="36" t="n"/>
+      <c r="Y18" s="36" t="n"/>
+      <c r="Z18" s="36" t="n"/>
+      <c r="AA18" s="36" t="n"/>
+      <c r="AB18" s="36" t="n"/>
+      <c r="AC18" s="36" t="n"/>
+      <c r="AD18" s="36" t="n"/>
+      <c r="AE18" s="36" t="n"/>
+      <c r="AF18" s="37" t="n"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>핵심 권한</t>
+        </is>
+      </c>
+      <c r="C19" s="36" t="n"/>
+      <c r="D19" s="36" t="n"/>
+      <c r="E19" s="36" t="n"/>
+      <c r="F19" s="36" t="n"/>
+      <c r="G19" s="36" t="n"/>
+      <c r="H19" s="36" t="n"/>
+      <c r="I19" s="37" t="n"/>
+      <c r="J19" s="34" t="inlineStr">
+        <is>
+          <t>작업중지 명령권, 협력업체 관리·감독권</t>
+        </is>
+      </c>
+      <c r="K19" s="36" t="n"/>
+      <c r="L19" s="36" t="n"/>
+      <c r="M19" s="36" t="n"/>
+      <c r="N19" s="36" t="n"/>
+      <c r="O19" s="36" t="n"/>
+      <c r="P19" s="36" t="n"/>
+      <c r="Q19" s="36" t="n"/>
+      <c r="R19" s="36" t="n"/>
+      <c r="S19" s="37" t="n"/>
+      <c r="T19" s="34" t="inlineStr">
+        <is>
+          <t>작업중지 요청권, 관리감독자 지도·조언권</t>
+        </is>
+      </c>
+      <c r="U19" s="36" t="n"/>
+      <c r="V19" s="36" t="n"/>
+      <c r="W19" s="36" t="n"/>
+      <c r="X19" s="36" t="n"/>
+      <c r="Y19" s="36" t="n"/>
+      <c r="Z19" s="36" t="n"/>
+      <c r="AA19" s="36" t="n"/>
+      <c r="AB19" s="36" t="n"/>
+      <c r="AC19" s="36" t="n"/>
+      <c r="AD19" s="36" t="n"/>
+      <c r="AE19" s="36" t="n"/>
+      <c r="AF19" s="37" t="n"/>
+    </row>
+    <row r="20" ht="12" customHeight="1"/>
+    <row r="21" ht="16" customHeight="1">
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>※ 근거: 산업안전보건법 제15조(안전보건관리책임자), 제17조(안전관리자), 제18조(안전관리자 등의 지도·조언), 중대재해처벌법 시행령 제4조(안전보건관리체계 구축·이행 점검)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="H7:AF7"/>
+    <mergeCell ref="B10:AF10"/>
+    <mergeCell ref="T17:AF17"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="H13:AF13"/>
+    <mergeCell ref="T16:AF16"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="H12:AF12"/>
+    <mergeCell ref="T19:AF19"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="J18:S18"/>
+    <mergeCell ref="B15:AF15"/>
+    <mergeCell ref="T18:AF18"/>
+    <mergeCell ref="B5:AF5"/>
+    <mergeCell ref="J17:S17"/>
+    <mergeCell ref="H8:AF8"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="J19:S19"/>
+    <mergeCell ref="B3:AF3"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B21:AF21"/>
+    <mergeCell ref="H6:AF6"/>
+    <mergeCell ref="B2:AF2"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="H11:AF11"/>
+    <mergeCell ref="J16:S16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF305496"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:AH13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="3" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="3" customWidth="1" min="9" max="9"/>
+    <col width="3" customWidth="1" min="10" max="10"/>
+    <col width="3" customWidth="1" min="11" max="11"/>
+    <col width="3" customWidth="1" min="12" max="12"/>
+    <col width="3" customWidth="1" min="13" max="13"/>
+    <col width="3" customWidth="1" min="14" max="14"/>
+    <col width="3" customWidth="1" min="15" max="15"/>
+    <col width="3" customWidth="1" min="16" max="16"/>
+    <col width="3" customWidth="1" min="17" max="17"/>
+    <col width="3" customWidth="1" min="18" max="18"/>
+    <col width="3" customWidth="1" min="19" max="19"/>
+    <col width="3" customWidth="1" min="20" max="20"/>
+    <col width="3" customWidth="1" min="21" max="21"/>
+    <col width="3" customWidth="1" min="22" max="22"/>
+    <col width="3" customWidth="1" min="23" max="23"/>
+    <col width="3" customWidth="1" min="24" max="24"/>
+    <col width="3" customWidth="1" min="25" max="25"/>
+    <col width="3" customWidth="1" min="26" max="26"/>
+    <col width="3" customWidth="1" min="27" max="27"/>
+    <col width="3" customWidth="1" min="28" max="28"/>
+    <col width="3" customWidth="1" min="29" max="29"/>
+    <col width="3" customWidth="1" min="30" max="30"/>
+    <col width="3" customWidth="1" min="31" max="31"/>
+    <col width="3" customWidth="1" min="32" max="32"/>
+    <col width="3" customWidth="1" min="33" max="33"/>
+    <col width="3" customWidth="1" min="34" max="34"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="6" customHeight="1"/>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>경영책임자 현장순회점검 시 3자 역할 비교</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
@@ -1407,127 +2053,159 @@
       <c r="AD2" s="2" t="n"/>
       <c r="AE2" s="2" t="n"/>
       <c r="AF2" s="2" t="n"/>
+      <c r="AG2" s="2" t="n"/>
+      <c r="AH2" s="2" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>(현장소장(안전보건관리책임자) 및 안전관리자 - 산업안전보건법 제15조·제17조, 중대재해처벌법 시행령 제4조 기준)</t>
+          <t>(안전보건관리책임자 · 안전관리자 · 관리감독자 - 산업안전보건법 제15조·제16조·제17조 기준)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="10" customHeight="1"/>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>1. 현장소장 (안전보건관리책임자) - 현장 총괄·최종 의사결정자</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-      <c r="P5" s="5" t="n"/>
-      <c r="Q5" s="5" t="n"/>
-      <c r="R5" s="5" t="n"/>
-      <c r="S5" s="5" t="n"/>
-      <c r="T5" s="5" t="n"/>
-      <c r="U5" s="5" t="n"/>
-      <c r="V5" s="5" t="n"/>
-      <c r="W5" s="5" t="n"/>
-      <c r="X5" s="5" t="n"/>
-      <c r="Y5" s="5" t="n"/>
-      <c r="Z5" s="5" t="n"/>
-      <c r="AA5" s="5" t="n"/>
-      <c r="AB5" s="5" t="n"/>
-      <c r="AC5" s="5" t="n"/>
-      <c r="AD5" s="5" t="n"/>
-      <c r="AE5" s="5" t="n"/>
-      <c r="AF5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="27" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="28" t="n"/>
-      <c r="E6" s="28" t="n"/>
-      <c r="F6" s="28" t="n"/>
-      <c r="G6" s="28" t="n"/>
-      <c r="H6" s="27" t="inlineStr">
-        <is>
-          <t>내용</t>
-        </is>
-      </c>
-      <c r="I6" s="28" t="n"/>
-      <c r="J6" s="28" t="n"/>
-      <c r="K6" s="28" t="n"/>
-      <c r="L6" s="28" t="n"/>
-      <c r="M6" s="28" t="n"/>
-      <c r="N6" s="28" t="n"/>
-      <c r="O6" s="28" t="n"/>
-      <c r="P6" s="28" t="n"/>
-      <c r="Q6" s="28" t="n"/>
-      <c r="R6" s="28" t="n"/>
-      <c r="S6" s="28" t="n"/>
-      <c r="T6" s="28" t="n"/>
-      <c r="U6" s="28" t="n"/>
-      <c r="V6" s="28" t="n"/>
-      <c r="W6" s="28" t="n"/>
-      <c r="X6" s="28" t="n"/>
-      <c r="Y6" s="28" t="n"/>
-      <c r="Z6" s="28" t="n"/>
-      <c r="AA6" s="28" t="n"/>
-      <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="28" t="n"/>
-      <c r="AD6" s="28" t="n"/>
-      <c r="AE6" s="28" t="n"/>
-      <c r="AF6" s="28" t="n"/>
-    </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="B7" s="29" t="inlineStr">
-        <is>
-          <t>책임</t>
+      <c r="C5" s="39" t="n"/>
+      <c r="D5" s="39" t="n"/>
+      <c r="E5" s="39" t="n"/>
+      <c r="F5" s="39" t="n"/>
+      <c r="G5" s="38" t="inlineStr">
+        <is>
+          <t>안전보건관리책임자
+(현장소장)</t>
+        </is>
+      </c>
+      <c r="H5" s="39" t="n"/>
+      <c r="I5" s="39" t="n"/>
+      <c r="J5" s="39" t="n"/>
+      <c r="K5" s="39" t="n"/>
+      <c r="L5" s="39" t="n"/>
+      <c r="M5" s="39" t="n"/>
+      <c r="N5" s="39" t="n"/>
+      <c r="O5" s="38" t="inlineStr">
+        <is>
+          <t>안전관리자</t>
+        </is>
+      </c>
+      <c r="P5" s="39" t="n"/>
+      <c r="Q5" s="39" t="n"/>
+      <c r="R5" s="39" t="n"/>
+      <c r="S5" s="39" t="n"/>
+      <c r="T5" s="39" t="n"/>
+      <c r="U5" s="39" t="n"/>
+      <c r="V5" s="38" t="inlineStr">
+        <is>
+          <t>관리감독자</t>
+        </is>
+      </c>
+      <c r="W5" s="39" t="n"/>
+      <c r="X5" s="39" t="n"/>
+      <c r="Y5" s="39" t="n"/>
+      <c r="Z5" s="39" t="n"/>
+      <c r="AA5" s="39" t="n"/>
+      <c r="AB5" s="39" t="n"/>
+      <c r="AC5" s="39" t="n"/>
+      <c r="AD5" s="39" t="n"/>
+      <c r="AE5" s="39" t="n"/>
+      <c r="AF5" s="39" t="n"/>
+      <c r="AG5" s="39" t="n"/>
+      <c r="AH5" s="39" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>위치·범위</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="30" t="n"/>
+      <c r="F6" s="30" t="n"/>
+      <c r="G6" s="40" t="inlineStr">
+        <is>
+          <t>현장 전체 총괄 · 최종 의사결정자</t>
+        </is>
+      </c>
+      <c r="H6" s="32" t="n"/>
+      <c r="I6" s="32" t="n"/>
+      <c r="J6" s="32" t="n"/>
+      <c r="K6" s="32" t="n"/>
+      <c r="L6" s="32" t="n"/>
+      <c r="M6" s="32" t="n"/>
+      <c r="N6" s="32" t="n"/>
+      <c r="O6" s="40" t="inlineStr">
+        <is>
+          <t>현장 전체(통합) 기술 전문가 · 보좌기관</t>
+        </is>
+      </c>
+      <c r="P6" s="32" t="n"/>
+      <c r="Q6" s="32" t="n"/>
+      <c r="R6" s="32" t="n"/>
+      <c r="S6" s="32" t="n"/>
+      <c r="T6" s="32" t="n"/>
+      <c r="U6" s="32" t="n"/>
+      <c r="V6" s="40" t="inlineStr">
+        <is>
+          <t>담당 공정 · 작업구역(부분) 실무 책임자</t>
+        </is>
+      </c>
+      <c r="W6" s="32" t="n"/>
+      <c r="X6" s="32" t="n"/>
+      <c r="Y6" s="32" t="n"/>
+      <c r="Z6" s="32" t="n"/>
+      <c r="AA6" s="32" t="n"/>
+      <c r="AB6" s="32" t="n"/>
+      <c r="AC6" s="32" t="n"/>
+      <c r="AD6" s="32" t="n"/>
+      <c r="AE6" s="32" t="n"/>
+      <c r="AF6" s="32" t="n"/>
+      <c r="AG6" s="32" t="n"/>
+      <c r="AH6" s="32" t="n"/>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>순회점검 시
+역할</t>
         </is>
       </c>
       <c r="C7" s="30" t="n"/>
       <c r="D7" s="30" t="n"/>
       <c r="E7" s="30" t="n"/>
       <c r="F7" s="30" t="n"/>
-      <c r="G7" s="30" t="n"/>
-      <c r="H7" s="31" t="inlineStr">
-        <is>
-          <t>- 현장 전체 안전보건관리에 대한 총괄 책임 - 순회점검 시 안전보건관리체계 이행현황(위험성평가, 교육, 관리비 집행 등)을 사실대로 보고
-- 점검 중 지적된 위험요인·미비사항에 대한 시정조치 및 재발방지대책 수립·이행
-- 점검결과에 따른 후속조치 이행 여부를 경영책임자에게 사후 보고
-- 근로자 의견청취 결과를 안전보건관리체계에 반영
-- 협력업체(수급인) 포함 현장 전체의 산업안전보건법 제15조 법정업무 이행</t>
-        </is>
-      </c>
+      <c r="G7" s="40" t="inlineStr">
+        <is>
+          <t>전체 현황 보고 + 최종 책임자로서 수검 대응</t>
+        </is>
+      </c>
+      <c r="H7" s="32" t="n"/>
       <c r="I7" s="32" t="n"/>
       <c r="J7" s="32" t="n"/>
       <c r="K7" s="32" t="n"/>
       <c r="L7" s="32" t="n"/>
       <c r="M7" s="32" t="n"/>
       <c r="N7" s="32" t="n"/>
-      <c r="O7" s="32" t="n"/>
+      <c r="O7" s="40" t="inlineStr">
+        <is>
+          <t>점검 동행, 전문자료 준비·설명, 관리감독자 총괄 지도</t>
+        </is>
+      </c>
       <c r="P7" s="32" t="n"/>
       <c r="Q7" s="32" t="n"/>
       <c r="R7" s="32" t="n"/>
       <c r="S7" s="32" t="n"/>
       <c r="T7" s="32" t="n"/>
       <c r="U7" s="32" t="n"/>
-      <c r="V7" s="32" t="n"/>
+      <c r="V7" s="40" t="inlineStr">
+        <is>
+          <t>담당 구역 현장답변, 즉시조치 실행</t>
+        </is>
+      </c>
       <c r="W7" s="32" t="n"/>
       <c r="X7" s="32" t="n"/>
       <c r="Y7" s="32" t="n"/>
@@ -1538,41 +2216,51 @@
       <c r="AD7" s="32" t="n"/>
       <c r="AE7" s="32" t="n"/>
       <c r="AF7" s="32" t="n"/>
-    </row>
-    <row r="8" ht="80" customHeight="1">
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>권한</t>
+      <c r="AG7" s="32" t="n"/>
+      <c r="AH7" s="32" t="n"/>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>설명·보고
+내용</t>
         </is>
       </c>
       <c r="C8" s="30" t="n"/>
       <c r="D8" s="30" t="n"/>
       <c r="E8" s="30" t="n"/>
       <c r="F8" s="30" t="n"/>
-      <c r="G8" s="30" t="n"/>
-      <c r="H8" s="31" t="inlineStr">
-        <is>
-          <t>- 현장 내 안전보건 관련 사항에 대한 최종 의사결정권
-- 위험 발생·우려 시 작업중지 명령권
-- 안전관리자 등 안전보건 인력에 대한 지휘·감독권
-- 협력업체에 대한 관리·감독 및 시정지시권
-- 안전보건관리비 집행 승인권</t>
-        </is>
-      </c>
+      <c r="G8" s="40" t="inlineStr">
+        <is>
+          <t>안전보건관리체계 이행현황 전반
+(위험성평가·교육·관리비 집행·조직운영 등)</t>
+        </is>
+      </c>
+      <c r="H8" s="32" t="n"/>
       <c r="I8" s="32" t="n"/>
       <c r="J8" s="32" t="n"/>
       <c r="K8" s="32" t="n"/>
       <c r="L8" s="32" t="n"/>
       <c r="M8" s="32" t="n"/>
       <c r="N8" s="32" t="n"/>
-      <c r="O8" s="32" t="n"/>
+      <c r="O8" s="40" t="inlineStr">
+        <is>
+          <t>위험성평가 결과, 안전장치·보호구 점검기록,
+재해통계 등 기술자료</t>
+        </is>
+      </c>
       <c r="P8" s="32" t="n"/>
       <c r="Q8" s="32" t="n"/>
       <c r="R8" s="32" t="n"/>
       <c r="S8" s="32" t="n"/>
       <c r="T8" s="32" t="n"/>
       <c r="U8" s="32" t="n"/>
-      <c r="V8" s="32" t="n"/>
+      <c r="V8" s="40" t="inlineStr">
+        <is>
+          <t>담당 공정 위험성평가·TBM 실시결과,
+소속 근로자 교육현황</t>
+        </is>
+      </c>
       <c r="W8" s="32" t="n"/>
       <c r="X8" s="32" t="n"/>
       <c r="Y8" s="32" t="n"/>
@@ -1583,433 +2271,209 @@
       <c r="AD8" s="32" t="n"/>
       <c r="AE8" s="32" t="n"/>
       <c r="AF8" s="32" t="n"/>
-    </row>
-    <row r="9" ht="12" customHeight="1"/>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>2. 안전관리자 - 기술 전문가·보좌기관</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="5" t="n"/>
-      <c r="P10" s="5" t="n"/>
-      <c r="Q10" s="5" t="n"/>
-      <c r="R10" s="5" t="n"/>
-      <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
-      <c r="U10" s="5" t="n"/>
-      <c r="V10" s="5" t="n"/>
-      <c r="W10" s="5" t="n"/>
-      <c r="X10" s="5" t="n"/>
-      <c r="Y10" s="5" t="n"/>
-      <c r="Z10" s="5" t="n"/>
-      <c r="AA10" s="5" t="n"/>
-      <c r="AB10" s="5" t="n"/>
-      <c r="AC10" s="5" t="n"/>
-      <c r="AD10" s="5" t="n"/>
-      <c r="AE10" s="5" t="n"/>
-      <c r="AF10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="B11" s="27" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="C11" s="28" t="n"/>
-      <c r="D11" s="28" t="n"/>
-      <c r="E11" s="28" t="n"/>
-      <c r="F11" s="28" t="n"/>
-      <c r="G11" s="28" t="n"/>
-      <c r="H11" s="27" t="inlineStr">
-        <is>
-          <t>내용</t>
-        </is>
-      </c>
-      <c r="I11" s="28" t="n"/>
-      <c r="J11" s="28" t="n"/>
-      <c r="K11" s="28" t="n"/>
-      <c r="L11" s="28" t="n"/>
-      <c r="M11" s="28" t="n"/>
-      <c r="N11" s="28" t="n"/>
-      <c r="O11" s="28" t="n"/>
-      <c r="P11" s="28" t="n"/>
-      <c r="Q11" s="28" t="n"/>
-      <c r="R11" s="28" t="n"/>
-      <c r="S11" s="28" t="n"/>
-      <c r="T11" s="28" t="n"/>
-      <c r="U11" s="28" t="n"/>
-      <c r="V11" s="28" t="n"/>
-      <c r="W11" s="28" t="n"/>
-      <c r="X11" s="28" t="n"/>
-      <c r="Y11" s="28" t="n"/>
-      <c r="Z11" s="28" t="n"/>
-      <c r="AA11" s="28" t="n"/>
-      <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="28" t="n"/>
-      <c r="AD11" s="28" t="n"/>
-      <c r="AE11" s="28" t="n"/>
-      <c r="AF11" s="28" t="n"/>
-    </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>책임</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="n"/>
-      <c r="D12" s="30" t="n"/>
-      <c r="E12" s="30" t="n"/>
-      <c r="F12" s="30" t="n"/>
-      <c r="G12" s="30" t="n"/>
-      <c r="H12" s="31" t="inlineStr">
-        <is>
-          <t>- 안전에 관한 기술적 사항에 대해 안전보건관리책임자를 보좌
-- 관리감독자에게 안전 관련 지도·조언
-- 순회점검 시 위험성평가 결과, 안전장치·보호구 점검현황, 아차사고/재해 통계 등 전문분야 자료 준비·설명
-- 지적사항 중 기술적 사항에 대한 개선방안 제시
-- 사업장 순회점검, 안전교육계획 수립, 산재 원인조사 등 법정 고유업무 수행(시행령 별표3)</t>
-        </is>
-      </c>
-      <c r="I12" s="32" t="n"/>
-      <c r="J12" s="32" t="n"/>
-      <c r="K12" s="32" t="n"/>
-      <c r="L12" s="32" t="n"/>
-      <c r="M12" s="32" t="n"/>
-      <c r="N12" s="32" t="n"/>
-      <c r="O12" s="32" t="n"/>
-      <c r="P12" s="32" t="n"/>
-      <c r="Q12" s="32" t="n"/>
-      <c r="R12" s="32" t="n"/>
-      <c r="S12" s="32" t="n"/>
-      <c r="T12" s="32" t="n"/>
-      <c r="U12" s="32" t="n"/>
-      <c r="V12" s="32" t="n"/>
-      <c r="W12" s="32" t="n"/>
-      <c r="X12" s="32" t="n"/>
-      <c r="Y12" s="32" t="n"/>
-      <c r="Z12" s="32" t="n"/>
-      <c r="AA12" s="32" t="n"/>
-      <c r="AB12" s="32" t="n"/>
-      <c r="AC12" s="32" t="n"/>
-      <c r="AD12" s="32" t="n"/>
-      <c r="AE12" s="32" t="n"/>
-      <c r="AF12" s="32" t="n"/>
-    </row>
-    <row r="13" ht="68" customHeight="1">
-      <c r="B13" s="29" t="inlineStr">
+      <c r="AG8" s="32" t="n"/>
+      <c r="AH8" s="32" t="n"/>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>지적사항
+대응</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="n"/>
+      <c r="D9" s="30" t="n"/>
+      <c r="E9" s="30" t="n"/>
+      <c r="F9" s="30" t="n"/>
+      <c r="G9" s="40" t="inlineStr">
+        <is>
+          <t>시정지시 결정 및 개선계획 수립,
+후속조치 총괄·본사 보고</t>
+        </is>
+      </c>
+      <c r="H9" s="32" t="n"/>
+      <c r="I9" s="32" t="n"/>
+      <c r="J9" s="32" t="n"/>
+      <c r="K9" s="32" t="n"/>
+      <c r="L9" s="32" t="n"/>
+      <c r="M9" s="32" t="n"/>
+      <c r="N9" s="32" t="n"/>
+      <c r="O9" s="40" t="inlineStr">
+        <is>
+          <t>근본원인 분석 및 기술적 개선방안 제시,
+작업중지 요청</t>
+        </is>
+      </c>
+      <c r="P9" s="32" t="n"/>
+      <c r="Q9" s="32" t="n"/>
+      <c r="R9" s="32" t="n"/>
+      <c r="S9" s="32" t="n"/>
+      <c r="T9" s="32" t="n"/>
+      <c r="U9" s="32" t="n"/>
+      <c r="V9" s="40" t="inlineStr">
+        <is>
+          <t>현장에서 즉시 시정조치
+(작업방법 개선, 표지 설치 등)</t>
+        </is>
+      </c>
+      <c r="W9" s="32" t="n"/>
+      <c r="X9" s="32" t="n"/>
+      <c r="Y9" s="32" t="n"/>
+      <c r="Z9" s="32" t="n"/>
+      <c r="AA9" s="32" t="n"/>
+      <c r="AB9" s="32" t="n"/>
+      <c r="AC9" s="32" t="n"/>
+      <c r="AD9" s="32" t="n"/>
+      <c r="AE9" s="32" t="n"/>
+      <c r="AF9" s="32" t="n"/>
+      <c r="AG9" s="32" t="n"/>
+      <c r="AH9" s="32" t="n"/>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>권한</t>
         </is>
       </c>
-      <c r="C13" s="30" t="n"/>
-      <c r="D13" s="30" t="n"/>
-      <c r="E13" s="30" t="n"/>
-      <c r="F13" s="30" t="n"/>
-      <c r="G13" s="30" t="n"/>
-      <c r="H13" s="31" t="inlineStr">
-        <is>
-          <t>- 위험 발견 시 안전보건관리책임자(또는 사업주)에게 작업중지 요청권
-- 관리감독자에 대한 지도·조언권
-- 안전보건 관련 자료 열람 및 시정요구권
-- 업무수행에 필요한 권한·시설·장비를 사업주로부터 지원받을 권리(법 제18조 - 독립적 업무수행 보장)</t>
-        </is>
-      </c>
-      <c r="I13" s="32" t="n"/>
-      <c r="J13" s="32" t="n"/>
-      <c r="K13" s="32" t="n"/>
-      <c r="L13" s="32" t="n"/>
-      <c r="M13" s="32" t="n"/>
-      <c r="N13" s="32" t="n"/>
-      <c r="O13" s="32" t="n"/>
-      <c r="P13" s="32" t="n"/>
-      <c r="Q13" s="32" t="n"/>
-      <c r="R13" s="32" t="n"/>
-      <c r="S13" s="32" t="n"/>
-      <c r="T13" s="32" t="n"/>
-      <c r="U13" s="32" t="n"/>
-      <c r="V13" s="32" t="n"/>
-      <c r="W13" s="32" t="n"/>
-      <c r="X13" s="32" t="n"/>
-      <c r="Y13" s="32" t="n"/>
-      <c r="Z13" s="32" t="n"/>
-      <c r="AA13" s="32" t="n"/>
-      <c r="AB13" s="32" t="n"/>
-      <c r="AC13" s="32" t="n"/>
-      <c r="AD13" s="32" t="n"/>
-      <c r="AE13" s="32" t="n"/>
-      <c r="AF13" s="32" t="n"/>
-    </row>
-    <row r="14" ht="12" customHeight="1"/>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>3. 핵심 비교</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-      <c r="L15" s="5" t="n"/>
-      <c r="M15" s="5" t="n"/>
-      <c r="N15" s="5" t="n"/>
-      <c r="O15" s="5" t="n"/>
-      <c r="P15" s="5" t="n"/>
-      <c r="Q15" s="5" t="n"/>
-      <c r="R15" s="5" t="n"/>
-      <c r="S15" s="5" t="n"/>
-      <c r="T15" s="5" t="n"/>
-      <c r="U15" s="5" t="n"/>
-      <c r="V15" s="5" t="n"/>
-      <c r="W15" s="5" t="n"/>
-      <c r="X15" s="5" t="n"/>
-      <c r="Y15" s="5" t="n"/>
-      <c r="Z15" s="5" t="n"/>
-      <c r="AA15" s="5" t="n"/>
-      <c r="AB15" s="5" t="n"/>
-      <c r="AC15" s="5" t="n"/>
-      <c r="AD15" s="5" t="n"/>
-      <c r="AE15" s="5" t="n"/>
-      <c r="AF15" s="5" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="27" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="C16" s="28" t="n"/>
-      <c r="D16" s="28" t="n"/>
-      <c r="E16" s="28" t="n"/>
-      <c r="F16" s="28" t="n"/>
-      <c r="G16" s="28" t="n"/>
-      <c r="H16" s="28" t="n"/>
-      <c r="I16" s="28" t="n"/>
-      <c r="J16" s="27" t="inlineStr">
-        <is>
-          <t>현장소장(안전보건관리책임자)</t>
-        </is>
-      </c>
-      <c r="K16" s="28" t="n"/>
-      <c r="L16" s="28" t="n"/>
-      <c r="M16" s="28" t="n"/>
-      <c r="N16" s="28" t="n"/>
-      <c r="O16" s="28" t="n"/>
-      <c r="P16" s="28" t="n"/>
-      <c r="Q16" s="28" t="n"/>
-      <c r="R16" s="28" t="n"/>
-      <c r="S16" s="28" t="n"/>
-      <c r="T16" s="27" t="inlineStr">
-        <is>
-          <t>안전관리자</t>
-        </is>
-      </c>
-      <c r="U16" s="28" t="n"/>
-      <c r="V16" s="28" t="n"/>
-      <c r="W16" s="28" t="n"/>
-      <c r="X16" s="28" t="n"/>
-      <c r="Y16" s="28" t="n"/>
-      <c r="Z16" s="28" t="n"/>
-      <c r="AA16" s="28" t="n"/>
-      <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="28" t="n"/>
-      <c r="AD16" s="28" t="n"/>
-      <c r="AE16" s="28" t="n"/>
-      <c r="AF16" s="28" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>성격</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="n"/>
-      <c r="D17" s="30" t="n"/>
-      <c r="E17" s="30" t="n"/>
-      <c r="F17" s="30" t="n"/>
-      <c r="G17" s="30" t="n"/>
-      <c r="H17" s="30" t="n"/>
-      <c r="I17" s="30" t="n"/>
-      <c r="J17" s="34" t="inlineStr">
-        <is>
-          <t>현장 총괄·최종 의사결정자</t>
-        </is>
-      </c>
-      <c r="K17" s="32" t="n"/>
-      <c r="L17" s="32" t="n"/>
-      <c r="M17" s="32" t="n"/>
-      <c r="N17" s="32" t="n"/>
-      <c r="O17" s="32" t="n"/>
-      <c r="P17" s="32" t="n"/>
-      <c r="Q17" s="32" t="n"/>
-      <c r="R17" s="32" t="n"/>
-      <c r="S17" s="32" t="n"/>
-      <c r="T17" s="34" t="inlineStr">
-        <is>
-          <t>기술 전문가·보좌기관</t>
-        </is>
-      </c>
-      <c r="U17" s="32" t="n"/>
-      <c r="V17" s="32" t="n"/>
-      <c r="W17" s="32" t="n"/>
-      <c r="X17" s="32" t="n"/>
-      <c r="Y17" s="32" t="n"/>
-      <c r="Z17" s="32" t="n"/>
-      <c r="AA17" s="32" t="n"/>
-      <c r="AB17" s="32" t="n"/>
-      <c r="AC17" s="32" t="n"/>
-      <c r="AD17" s="32" t="n"/>
-      <c r="AE17" s="32" t="n"/>
-      <c r="AF17" s="32" t="n"/>
-    </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>순회점검 역할</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="n"/>
-      <c r="D18" s="30" t="n"/>
-      <c r="E18" s="30" t="n"/>
-      <c r="F18" s="30" t="n"/>
-      <c r="G18" s="30" t="n"/>
-      <c r="H18" s="30" t="n"/>
-      <c r="I18" s="30" t="n"/>
-      <c r="J18" s="34" t="inlineStr">
-        <is>
-          <t>전체 현황 보고 + 최종 책임</t>
-        </is>
-      </c>
-      <c r="K18" s="32" t="n"/>
-      <c r="L18" s="32" t="n"/>
-      <c r="M18" s="32" t="n"/>
-      <c r="N18" s="32" t="n"/>
-      <c r="O18" s="32" t="n"/>
-      <c r="P18" s="32" t="n"/>
-      <c r="Q18" s="32" t="n"/>
-      <c r="R18" s="32" t="n"/>
-      <c r="S18" s="32" t="n"/>
-      <c r="T18" s="34" t="inlineStr">
-        <is>
-          <t>전문분야(위험성평가·점검기록) 설명 + 기술적 개선안 제시</t>
-        </is>
-      </c>
-      <c r="U18" s="32" t="n"/>
-      <c r="V18" s="32" t="n"/>
-      <c r="W18" s="32" t="n"/>
-      <c r="X18" s="32" t="n"/>
-      <c r="Y18" s="32" t="n"/>
-      <c r="Z18" s="32" t="n"/>
-      <c r="AA18" s="32" t="n"/>
-      <c r="AB18" s="32" t="n"/>
-      <c r="AC18" s="32" t="n"/>
-      <c r="AD18" s="32" t="n"/>
-      <c r="AE18" s="32" t="n"/>
-      <c r="AF18" s="32" t="n"/>
-    </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>핵심 권한</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="n"/>
-      <c r="D19" s="30" t="n"/>
-      <c r="E19" s="30" t="n"/>
-      <c r="F19" s="30" t="n"/>
-      <c r="G19" s="30" t="n"/>
-      <c r="H19" s="30" t="n"/>
-      <c r="I19" s="30" t="n"/>
-      <c r="J19" s="34" t="inlineStr">
-        <is>
-          <t>작업중지 명령권, 협력업체 관리·감독권</t>
-        </is>
-      </c>
-      <c r="K19" s="32" t="n"/>
-      <c r="L19" s="32" t="n"/>
-      <c r="M19" s="32" t="n"/>
-      <c r="N19" s="32" t="n"/>
-      <c r="O19" s="32" t="n"/>
-      <c r="P19" s="32" t="n"/>
-      <c r="Q19" s="32" t="n"/>
-      <c r="R19" s="32" t="n"/>
-      <c r="S19" s="32" t="n"/>
-      <c r="T19" s="34" t="inlineStr">
-        <is>
-          <t>작업중지 요청권, 관리감독자 지도·조언권</t>
-        </is>
-      </c>
-      <c r="U19" s="32" t="n"/>
-      <c r="V19" s="32" t="n"/>
-      <c r="W19" s="32" t="n"/>
-      <c r="X19" s="32" t="n"/>
-      <c r="Y19" s="32" t="n"/>
-      <c r="Z19" s="32" t="n"/>
-      <c r="AA19" s="32" t="n"/>
-      <c r="AB19" s="32" t="n"/>
-      <c r="AC19" s="32" t="n"/>
-      <c r="AD19" s="32" t="n"/>
-      <c r="AE19" s="32" t="n"/>
-      <c r="AF19" s="32" t="n"/>
-    </row>
-    <row r="20" ht="12" customHeight="1"/>
-    <row r="21" ht="16" customHeight="1">
-      <c r="B21" s="35" t="inlineStr">
-        <is>
-          <t>※ 근거: 산업안전보건법 제15조(안전보건관리책임자), 제17조(안전관리자), 제18조(안전관리자 등의 지도·조언), 중대재해처벌법 시행령 제4조(안전보건관리체계 구축·이행 점검)</t>
+      <c r="C10" s="30" t="n"/>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="30" t="n"/>
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="40" t="inlineStr">
+        <is>
+          <t>최종 의사결정권, 작업중지 명령권,
+협력업체 관리·감독권</t>
+        </is>
+      </c>
+      <c r="H10" s="32" t="n"/>
+      <c r="I10" s="32" t="n"/>
+      <c r="J10" s="32" t="n"/>
+      <c r="K10" s="32" t="n"/>
+      <c r="L10" s="32" t="n"/>
+      <c r="M10" s="32" t="n"/>
+      <c r="N10" s="32" t="n"/>
+      <c r="O10" s="40" t="inlineStr">
+        <is>
+          <t>작업중지 요청권, 관리감독자 지도·조언권,
+자료 열람·시정요구권</t>
+        </is>
+      </c>
+      <c r="P10" s="32" t="n"/>
+      <c r="Q10" s="32" t="n"/>
+      <c r="R10" s="32" t="n"/>
+      <c r="S10" s="32" t="n"/>
+      <c r="T10" s="32" t="n"/>
+      <c r="U10" s="32" t="n"/>
+      <c r="V10" s="40" t="inlineStr">
+        <is>
+          <t>담당구역 작업방법 변경·일시중지 지시권</t>
+        </is>
+      </c>
+      <c r="W10" s="32" t="n"/>
+      <c r="X10" s="32" t="n"/>
+      <c r="Y10" s="32" t="n"/>
+      <c r="Z10" s="32" t="n"/>
+      <c r="AA10" s="32" t="n"/>
+      <c r="AB10" s="32" t="n"/>
+      <c r="AC10" s="32" t="n"/>
+      <c r="AD10" s="32" t="n"/>
+      <c r="AE10" s="32" t="n"/>
+      <c r="AF10" s="32" t="n"/>
+      <c r="AG10" s="32" t="n"/>
+      <c r="AH10" s="32" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>법적 근거</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="n"/>
+      <c r="D11" s="30" t="n"/>
+      <c r="E11" s="30" t="n"/>
+      <c r="F11" s="30" t="n"/>
+      <c r="G11" s="40" t="inlineStr">
+        <is>
+          <t>산업안전보건법 제15조</t>
+        </is>
+      </c>
+      <c r="H11" s="32" t="n"/>
+      <c r="I11" s="32" t="n"/>
+      <c r="J11" s="32" t="n"/>
+      <c r="K11" s="32" t="n"/>
+      <c r="L11" s="32" t="n"/>
+      <c r="M11" s="32" t="n"/>
+      <c r="N11" s="32" t="n"/>
+      <c r="O11" s="40" t="inlineStr">
+        <is>
+          <t>산업안전보건법 제17조·제18조</t>
+        </is>
+      </c>
+      <c r="P11" s="32" t="n"/>
+      <c r="Q11" s="32" t="n"/>
+      <c r="R11" s="32" t="n"/>
+      <c r="S11" s="32" t="n"/>
+      <c r="T11" s="32" t="n"/>
+      <c r="U11" s="32" t="n"/>
+      <c r="V11" s="40" t="inlineStr">
+        <is>
+          <t>산업안전보건법 제16조</t>
+        </is>
+      </c>
+      <c r="W11" s="32" t="n"/>
+      <c r="X11" s="32" t="n"/>
+      <c r="Y11" s="32" t="n"/>
+      <c r="Z11" s="32" t="n"/>
+      <c r="AA11" s="32" t="n"/>
+      <c r="AB11" s="32" t="n"/>
+      <c r="AC11" s="32" t="n"/>
+      <c r="AD11" s="32" t="n"/>
+      <c r="AE11" s="32" t="n"/>
+      <c r="AF11" s="32" t="n"/>
+      <c r="AG11" s="32" t="n"/>
+      <c r="AH11" s="32" t="n"/>
+    </row>
+    <row r="12" ht="12" customHeight="1"/>
+    <row r="13" ht="16" customHeight="1">
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>※ 요약: 안전보건관리책임자는 "총괄 보고·의사결정", 안전관리자는 "기술 설명·전체 조정", 관리감독자는 "담당구역 실무 답변·즉시조치"로 역할이 구분됨</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="H7:AF7"/>
-    <mergeCell ref="B10:AF10"/>
-    <mergeCell ref="T17:AF17"/>
-    <mergeCell ref="B16:I16"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="H13:AF13"/>
-    <mergeCell ref="T16:AF16"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="H12:AF12"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="T19:AF19"/>
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="J18:S18"/>
-    <mergeCell ref="B15:AF15"/>
-    <mergeCell ref="T18:AF18"/>
-    <mergeCell ref="B5:AF5"/>
-    <mergeCell ref="J17:S17"/>
-    <mergeCell ref="H8:AF8"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B17:I17"/>
-    <mergeCell ref="J19:S19"/>
-    <mergeCell ref="B3:AF3"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B21:AF21"/>
-    <mergeCell ref="H6:AF6"/>
-    <mergeCell ref="B2:AF2"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="H11:AF11"/>
-    <mergeCell ref="J16:S16"/>
+  <mergeCells count="31">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="O8:U8"/>
+    <mergeCell ref="G11:N11"/>
+    <mergeCell ref="B2:AH2"/>
+    <mergeCell ref="O11:U11"/>
+    <mergeCell ref="V7:AH7"/>
+    <mergeCell ref="G8:N8"/>
+    <mergeCell ref="B13:AH13"/>
+    <mergeCell ref="G7:N7"/>
+    <mergeCell ref="O7:U7"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G10:N10"/>
+    <mergeCell ref="O10:U10"/>
+    <mergeCell ref="G6:N6"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="O6:U6"/>
+    <mergeCell ref="V5:AH5"/>
+    <mergeCell ref="O9:U9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="V8:AH8"/>
+    <mergeCell ref="O5:U5"/>
+    <mergeCell ref="G5:N5"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="V10:AH10"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="V9:AH9"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="V6:AH6"/>
+    <mergeCell ref="B3:AH3"/>
+    <mergeCell ref="G9:N9"/>
+    <mergeCell ref="V11:AH11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>